<commit_message>
Reformat Sankar Mallick admission diagnosis & procedure to insurance summary style
All-caps block format matching the hospital's discharge summary layout
(diagnosis / examination / procedure paragraph ending with performed-by
line); detailed narrative retained below for hospital record.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YWgR3jd3MUcEXpU4s4WC54
</commit_message>
<xml_diff>
--- a/BKAditya_SankarMallick_MediclaimBill.xlsx
+++ b/BKAditya_SankarMallick_MediclaimBill.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -66,6 +66,11 @@
       <color rgb="00C00000"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <i val="1"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -111,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -151,6 +156,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1780,7 +1788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:A38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -1808,36 +1816,44 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="18" t="inlineStr"/>
+      <c r="A4" s="19" t="inlineStr">
+        <is>
+          <t>ADMISSION DIAGNOSIS</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="inlineStr">
-        <is>
-          <t>FINAL DIAGNOSIS</t>
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>OLD MALUNITED FRACTURE OF SHAFT OF RIGHT TIBIA WITH IMPLANT IN SITU WITH IMPLANT LOOSENING WITH SECONDARY STIFFNESS OF RIGHT KNEE JOINT -</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>Old malunited fracture, shaft of right tibia, with loosening of in-situ implant; secondary stiffness of the right knee joint.</t>
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>EXAMINATION  (fill vitals at admission)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="18" t="inlineStr"/>
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>PT A/C/C,  PR- ___/MIN ,BP- ___/___ MMHG,  SPO2- ___% @ R/A,  TEMP- AFEBRILE,  CBG- ___ MG/DL,</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="19" t="inlineStr">
         <is>
-          <t>PRESENTING HISTORY &amp; FINDINGS</t>
+          <t>PROCEDURE  (insurance format)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="18" t="inlineStr">
         <is>
-          <t>Patient presented with pain and deformity of the right leg over a previously operated fracture. X-rays of the right leg (AP/lateral) revealed an old malunited tibial fracture with implant in situ, radiological evidence of implant loosening (peri-implant lucency / backed-out screws), and associated stiffness of the right knee secondary to the malunion. Pre-anaesthetic check-up and baseline investigations (CBG documented) were within acceptable limits for surgery.</t>
+          <t>THE PATIENT WAS PLACED IN THE SUPINE POSITION. PAINT AND DRAPING WERE DONE UNDER SPINAL ANESTHESIA. UNDER TOURNIQUET CONTROL, THE PREVIOUS SURGICAL SCAR OVER THE RIGHT TIBIA WAS INCISED AND DEEPENED. THE IN-SITU LOOSENED TIBIAL IMPLANT [PLATE AND SCREWS / INTERLOCKING NAIL — CONFIRM] WAS EXPOSED, AND THE OVERLYING FIBROUS AND SCLEROTIC TISSUE WAS CLEARED. ALL SCREWS WERE REMOVED SEQUENTIALLY AND THE IMPLANT WAS EXTRACTED IN TOTO UNDER C-ARM (IMAGE INTENSIFIER) GUIDANCE. MAJOR BONE DEBRIDEMENT WAS PERFORMED — LOOSE/DEVITALISED BONE AND HYPERTROPHIC CALLUS AT THE MALUNION SITE WERE DEBRIDED BACK TO HEALTHY BLEEDING BONE, FOLLOWED BY THOROUGH SALINE LAVAGE. HEMOSTASIS WAS SECURED WITH DIATHERMY/CAUTERY. CLOSURE WAS DONE IN LAYERS WITH VICRYL NO. 1 (DEEP) AND ETHILON 2-0 (SKIN). GENTLE MANIPULATION UNDER ANESTHESIA (MUA) OF THE RIGHT KNEE WAS THEN PERFORMED TO RELEASE ADHESIONS, ACHIEVING IMPROVED RANGE OF MOTION. THE TOURNIQUET WAS RELEASED WITH GOOD DISTAL PERFUSION AND MINIMAL BLOOD LOSS. STERILE DRESSING AND CREPE BANDAGE WERE APPLIED, AND THE PATIENT WAS SHIFTED TO THE WARD IN A STABLE CONDITION. THIS PROCEDURE WAS PERFORMED BY DR. KESHAV DIGGA ON 02/07/2026.</t>
         </is>
       </c>
     </row>
@@ -1845,30 +1861,26 @@
       <c r="A10" s="18" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>PROCEDURE PERFORMED (02/07/2026, 6:50 PM – 7:40 PM)</t>
+      <c r="A11" s="21" t="inlineStr">
+        <is>
+          <t>——— Detailed narrative version below (same procedure, for hospital record) ———</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="inlineStr">
-        <is>
-          <t>MAJOR IMPLANT REMOVAL (RIGHT TIBIA) + MANIPULATION UNDER ANAESTHESIA (MUA) OF RIGHT KNEE + MAJOR BONE DEBRIDEMENT</t>
-        </is>
-      </c>
+      <c r="A12" s="18" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>Under all aseptic precautions, spinal anaesthesia (Inj. Anawin Heavy 0.75% via 25G spinal needle, administered by Dr. Rahuldeb Mondal) and tourniquet control, the right leg was painted with Betadine and draped. The previous surgical scar was incised and deepened; the in-situ tibial implant [plate and screws / interlocking nail — CONFIRM hardware removed] was exposed. Fibrous and sclerotic tissue overlying the implant was cleared. All screws were removed sequentially and the implant was extracted in toto under C-Arm (image intensifier) guidance. Loose/devitalised bone and hypertrophic callus at the malunion site were debrided back to healthy bleeding bone; the wound was given a thorough saline lavage. Haemostasis was achieved with diathermy/cautery. Closure was done in layers with Vicryl No. 1 (deep) and Ethilon 2-0 (skin). Sterile dressing and crepe bandage applied.</t>
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>FINAL DIAGNOSIS</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="18" t="inlineStr">
         <is>
-          <t>Following wound closure, gentle manipulation of the right knee was performed under the same anaesthesia to release adhesions, achieving improved range of motion [pre-MUA ____° → post-MUA ____° — CONFIRM]. No intra-operative complications; tourniquet released with good distal perfusion; minimal blood loss.</t>
+          <t>Old malunited fracture, shaft of right tibia, with loosening of in-situ implant; secondary stiffness of the right knee joint.</t>
         </is>
       </c>
     </row>
@@ -1878,14 +1890,14 @@
     <row r="16">
       <c r="A16" s="19" t="inlineStr">
         <is>
-          <t>POST-OPERATIVE COURSE IN HOSPITAL</t>
+          <t>PRESENTING HISTORY &amp; FINDINGS</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="18" t="inlineStr">
         <is>
-          <t>Uneventful. Patient was monitored (pulse oximeter, cardiac monitor) and managed with IV antibiotics (Inj. Ceftriaxone 1g), IV analgesics (Inj. Paracetamol 1g IV, Inj. Diclofenac, Inj. Tramadol), Inj. Pantoprazole, Inj. Ondansetron and IV fluids as per chart. Wound inspected on POD-2 — healthy, no discharge. Knee mobilisation and static quadriceps physiotherapy started from POD-1 as advised. Patient ambulated with partial weight bearing using walker support. Discharged on POD-4 in haemodynamically stable condition with wound healthy.</t>
+          <t>Patient presented with pain and deformity of the right leg over a previously operated fracture. X-rays of the right leg (AP/lateral) revealed an old malunited tibial fracture with implant in situ, radiological evidence of implant loosening (peri-implant lucency / backed-out screws), and associated stiffness of the right knee secondary to the malunion. Pre-anaesthetic check-up and baseline investigations (CBG documented) were within acceptable limits for surgery.</t>
         </is>
       </c>
     </row>
@@ -1895,58 +1907,62 @@
     <row r="19">
       <c r="A19" s="19" t="inlineStr">
         <is>
+          <t>PROCEDURE PERFORMED (02/07/2026, 6:50 PM – 7:40 PM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>MAJOR IMPLANT REMOVAL (RIGHT TIBIA) + MANIPULATION UNDER ANAESTHESIA (MUA) OF RIGHT KNEE + MAJOR BONE DEBRIDEMENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>Under all aseptic precautions, spinal anaesthesia (Inj. Anawin Heavy 0.75% via 25G spinal needle, administered by Dr. Rahuldeb Mondal) and tourniquet control, the right leg was painted with Betadine and draped. The previous surgical scar was incised and deepened; the in-situ tibial implant [plate and screws / interlocking nail — CONFIRM hardware removed] was exposed. Fibrous and sclerotic tissue overlying the implant was cleared. All screws were removed sequentially and the implant was extracted in toto under C-Arm (image intensifier) guidance. Loose/devitalised bone and hypertrophic callus at the malunion site were debrided back to healthy bleeding bone; the wound was given a thorough saline lavage. Haemostasis was achieved with diathermy/cautery. Closure was done in layers with Vicryl No. 1 (deep) and Ethilon 2-0 (skin). Sterile dressing and crepe bandage applied.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="18" t="inlineStr">
+        <is>
+          <t>Following wound closure, gentle manipulation of the right knee was performed under the same anaesthesia to release adhesions, achieving improved range of motion [pre-MUA ____° → post-MUA ____° — CONFIRM]. No intra-operative complications; tourniquet released with good distal perfusion; minimal blood loss.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="18" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>POST-OPERATIVE COURSE IN HOSPITAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>Uneventful. Patient was monitored (pulse oximeter, cardiac monitor) and managed with IV antibiotics (Inj. Ceftriaxone 1g), IV analgesics (Inj. Paracetamol 1g IV, Inj. Diclofenac, Inj. Tramadol), Inj. Pantoprazole, Inj. Ondansetron and IV fluids as per chart. Wound inspected on POD-2 — healthy, no discharge. Knee mobilisation and static quadriceps physiotherapy started from POD-1 as advised. Patient ambulated with partial weight bearing using walker support. Discharged on POD-4 in haemodynamically stable condition with wound healthy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="18" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="19" t="inlineStr">
+        <is>
           <t>CONDITION AT DISCHARGE</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="18" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="18" t="inlineStr">
         <is>
           <t>Afebrile, vitals stable, wound clean and dry, distal neurovascular status intact, pain controlled on oral medication.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="18" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="19" t="inlineStr">
-        <is>
-          <t>DISCHARGE MEDICATIONS</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="18" t="inlineStr">
-        <is>
-          <t>1. Tab. Cefuroxime 500mg BD × 5 days   2. Tab. Paracetamol 650mg TDS × 5 days   3. Tab. Pantoprazole 40mg OD × 10 days   4. Cap. Calcium + Vitamin D3 OD × 30 days   [adjust per consultant]</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="18" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="19" t="inlineStr">
-        <is>
-          <t>ADVICE ON DISCHARGE</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="18" t="inlineStr">
-        <is>
-          <t>• Partial weight bearing with walker for 2 weeks, then progressive full weight bearing as tolerated. • Continue knee ROM and quadriceps strengthening physiotherapy. • Keep wound dry; dressing change on alternate days. • Suture removal on POD-12/14 at OPD. • Review in OPD after 10 days with X-ray right leg, or earlier if fever, wound discharge, or increased pain.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="18" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="17" t="inlineStr">
-        <is>
-          <t>Dr. Keshav Digga, MS (Orthopaedics)                                    Signature: ____________________</t>
         </is>
       </c>
     </row>
@@ -1954,7 +1970,51 @@
       <c r="A29" s="18" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="20" t="inlineStr">
+      <c r="A30" s="19" t="inlineStr">
+        <is>
+          <t>DISCHARGE MEDICATIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="18" t="inlineStr">
+        <is>
+          <t>1. Tab. Cefuroxime 500mg BD × 5 days   2. Tab. Paracetamol 650mg TDS × 5 days   3. Tab. Pantoprazole 40mg OD × 10 days   4. Cap. Calcium + Vitamin D3 OD × 30 days   [adjust per consultant]</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="18" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="19" t="inlineStr">
+        <is>
+          <t>ADVICE ON DISCHARGE</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="18" t="inlineStr">
+        <is>
+          <t>• Partial weight bearing with walker for 2 weeks, then progressive full weight bearing as tolerated. • Continue knee ROM and quadriceps strengthening physiotherapy. • Keep wound dry; dressing change on alternate days. • Suture removal on POD-12/14 at OPD. • Review in OPD after 10 days with X-ray right leg, or earlier if fever, wound discharge, or increased pain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="18" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="17" t="inlineStr">
+        <is>
+          <t>Dr. Keshav Digga, MS (Orthopaedics)                                    Signature: ____________________</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="18" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="20" t="inlineStr">
         <is>
           <t>⚠ DRAFT: fields in [brackets] (hardware removed, knee ROM values, medication doses) must be confirmed/filled by the operating surgeon before this goes on hospital letterhead.</t>
         </is>

</xml_diff>